<commit_message>
Clean up generation script: remove dead code and misleading comments
Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/f32a1be0-decb-424d-a30d-a09190ff9301

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -216,6 +216,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -721,7 +722,7 @@
       </c>
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="5">
-        <f>SUM(C12:C23)</f>
+        <f>SUM(D12:D23)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="n"/>
@@ -735,7 +736,7 @@
       </c>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="5">
-        <f>SUM(D12:D23)</f>
+        <f>SUM(E12:E23)</f>
         <v/>
       </c>
       <c r="E6" s="4" t="n"/>
@@ -4090,7 +4091,9 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="B2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="B3" s="8" t="inlineStr">
         <is>
@@ -4112,7 +4115,9 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="B6" t="inlineStr"/>
+    </row>
     <row r="7">
       <c r="B7" s="8" t="inlineStr">
         <is>
@@ -4148,7 +4153,9 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
+    <row r="12">
+      <c r="B12" t="inlineStr"/>
+    </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -4184,7 +4191,9 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
+    <row r="18">
+      <c r="B18" t="inlineStr"/>
+    </row>
     <row r="19">
       <c r="B19" s="8" t="inlineStr">
         <is>
@@ -4213,7 +4222,9 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="23">
+      <c r="B23" t="inlineStr"/>
+    </row>
     <row r="24">
       <c r="B24" s="8" t="inlineStr">
         <is>
@@ -4249,7 +4260,9 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
+    <row r="29">
+      <c r="B29" t="inlineStr"/>
+    </row>
     <row r="30">
       <c r="B30" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add abundant icons throughout the spreadsheet for a catchy visual style
- Seasonal emojis for each month (⛄1月, 💝2月, 🌸3月, etc.)
- Category icons for income (💼給与, 🔨副業, 📈投資収入, 🎁その他)
- Category icons for expenses (🏠住居, 💡光熱, 🍽️食費, 🚃交通, etc.)
- Section headers with emojis (💚収入, 🔴支出, ⚖️収支バランス, 📝日別記録)
- Bills tracker with service icons (⚡電気, 🔥ガス, 💧水道, 🎬Netflix, etc.)
- Savings goals with icons (🆘緊急, ✈️旅行, 🚗車, 🎓教育, 🏖️老後)
- Table headers with icons throughout all sheets
- Instructions guide with emoji markers (1️⃣2️⃣3️⃣4️⃣, section icons)

Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/259d5db9-2402-4d23-ab8c-32e8bfbacec0

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -1035,59 +1035,59 @@
       <c r="A9" s="14" t="n"/>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>🗓️ 月</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>収入</t>
+          <t>💚 収入</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>支出</t>
+          <t>🔴 支出</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>貯蓄</t>
+          <t>💰 貯蓄</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>貯蓄率</t>
+          <t>📊 貯蓄率</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>前月比支出</t>
+          <t>📉 前月比支出</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>評価</t>
+          <t>🏅 評価</t>
         </is>
       </c>
       <c r="J9" s="15" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>年間合計</t>
+          <t>💴 年間合計</t>
         </is>
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>構成比</t>
+          <t>📊 構成比</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>1月</t>
+          <t>⛄ 1月</t>
         </is>
       </c>
       <c r="C10" s="17">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="K10" s="17">
@@ -1131,7 +1131,7 @@
     <row r="11">
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>2月</t>
+          <t>💝 2月</t>
         </is>
       </c>
       <c r="C11" s="23">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="J11" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="K11" s="23">
@@ -1175,7 +1175,7 @@
     <row r="12">
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>3月</t>
+          <t>🌸 3月</t>
         </is>
       </c>
       <c r="C12" s="17">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J12" s="19" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="K12" s="17">
@@ -1219,7 +1219,7 @@
     <row r="13">
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>4月</t>
+          <t>🌷 4月</t>
         </is>
       </c>
       <c r="C13" s="23">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="J13" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="K13" s="23">
@@ -1263,7 +1263,7 @@
     <row r="14">
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>🎏 5月</t>
         </is>
       </c>
       <c r="C14" s="17">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="K14" s="17">
@@ -1307,7 +1307,7 @@
     <row r="15">
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>☔ 6月</t>
         </is>
       </c>
       <c r="C15" s="23">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="J15" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="K15" s="23">
@@ -1351,7 +1351,7 @@
     <row r="16">
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>🎋 7月</t>
         </is>
       </c>
       <c r="C16" s="17">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="K16" s="17">
@@ -1395,7 +1395,7 @@
     <row r="17">
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>🌻 8月</t>
         </is>
       </c>
       <c r="C17" s="23">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J17" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="K17" s="23">
@@ -1439,7 +1439,7 @@
     <row r="18">
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>🌾 9月</t>
         </is>
       </c>
       <c r="C18" s="17">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="K18" s="17">
@@ -1483,7 +1483,7 @@
     <row r="19">
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>10月</t>
+          <t>🎃 10月</t>
         </is>
       </c>
       <c r="C19" s="23">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="J19" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="K19" s="23">
@@ -1527,7 +1527,7 @@
     <row r="20">
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>11月</t>
+          <t>🍂 11月</t>
         </is>
       </c>
       <c r="C20" s="17">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="J20" s="19" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="K20" s="17">
@@ -1571,7 +1571,7 @@
     <row r="21">
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>12月</t>
+          <t>🎄 12月</t>
         </is>
       </c>
       <c r="C21" s="23">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="J21" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="K21" s="23">
@@ -1615,7 +1615,7 @@
     <row r="22">
       <c r="J22" s="19" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="K22" s="17">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="J23" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="K23" s="23">
@@ -1691,14 +1691,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 9月 家計簿</t>
+          <t>🌾 9月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -1709,7 +1709,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -1724,7 +1724,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -1739,7 +1739,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -1754,7 +1754,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -1769,7 +1769,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -1780,7 +1780,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -1795,7 +1795,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -1810,7 +1810,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -1825,7 +1825,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -1840,7 +1840,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -1855,7 +1855,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -1870,7 +1870,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -1885,7 +1885,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -1900,7 +1900,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -1915,7 +1915,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -1930,7 +1930,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -1945,7 +1945,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -1960,7 +1960,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -1975,7 +1975,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -1990,14 +1990,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -2008,7 +2008,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -2019,7 +2019,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -2030,7 +2030,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -2038,27 +2038,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -2308,14 +2308,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 10月 家計簿</t>
+          <t>🎃 10月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -2326,7 +2326,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -2341,7 +2341,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -2356,7 +2356,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -2371,7 +2371,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -2386,7 +2386,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -2397,7 +2397,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -2412,7 +2412,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -2427,7 +2427,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -2442,7 +2442,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -2457,7 +2457,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -2472,7 +2472,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -2487,7 +2487,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -2502,7 +2502,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -2517,7 +2517,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -2532,7 +2532,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -2547,7 +2547,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -2562,7 +2562,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -2577,7 +2577,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -2592,7 +2592,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -2607,14 +2607,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -2625,7 +2625,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -2636,7 +2636,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -2647,7 +2647,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -2655,27 +2655,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -2925,14 +2925,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 11月 家計簿</t>
+          <t>🍂 11月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -2943,7 +2943,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -2958,7 +2958,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -2973,7 +2973,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -2988,7 +2988,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -3003,7 +3003,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -3014,7 +3014,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -3029,7 +3029,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -3044,7 +3044,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -3059,7 +3059,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -3074,7 +3074,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -3089,7 +3089,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -3104,7 +3104,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -3119,7 +3119,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -3134,7 +3134,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -3149,7 +3149,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -3164,7 +3164,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -3179,7 +3179,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -3194,7 +3194,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -3209,7 +3209,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -3224,14 +3224,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -3242,7 +3242,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -3253,7 +3253,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -3264,7 +3264,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -3272,27 +3272,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -3542,14 +3542,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 12月 家計簿</t>
+          <t>🎄 12月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -3560,7 +3560,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -3575,7 +3575,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -3590,7 +3590,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -3605,7 +3605,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -3620,7 +3620,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -3631,7 +3631,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -3646,7 +3646,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -3661,7 +3661,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -3676,7 +3676,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -3691,7 +3691,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -3706,7 +3706,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -3721,7 +3721,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -3736,7 +3736,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -3751,7 +3751,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -3766,7 +3766,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -3781,7 +3781,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -3796,7 +3796,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -3811,7 +3811,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -3826,7 +3826,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -3841,14 +3841,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -3859,7 +3859,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -3870,7 +3870,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -3881,7 +3881,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -3889,27 +3889,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -4168,44 +4168,44 @@
       <c r="A3" s="14" t="n"/>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>項目名</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>月額</t>
+          <t>💴 月額</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>支払日</t>
+          <t>📅 支払日</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F3" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>次回支払日</t>
+          <t>⏰ 次回支払日</t>
         </is>
       </c>
       <c r="H3" s="14" t="inlineStr">
         <is>
-          <t>ステータス</t>
+          <t>✅ ステータス</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>家賃</t>
+          <t>🏠 家賃</t>
         </is>
       </c>
       <c r="C4" s="23" t="n">
@@ -4230,7 +4230,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>電気代</t>
+          <t>⚡ 電気代</t>
         </is>
       </c>
       <c r="C5" s="23" t="n">
@@ -4255,7 +4255,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>ガス代</t>
+          <t>🔥 ガス代</t>
         </is>
       </c>
       <c r="C6" s="23" t="n">
@@ -4280,7 +4280,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>水道代</t>
+          <t>💧 水道代</t>
         </is>
       </c>
       <c r="C7" s="23" t="n">
@@ -4305,7 +4305,7 @@
     <row r="8">
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>携帯電話</t>
+          <t>📱 携帯電話</t>
         </is>
       </c>
       <c r="C8" s="23" t="n">
@@ -4330,7 +4330,7 @@
     <row r="9">
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>インターネット</t>
+          <t>🌐 インターネット</t>
         </is>
       </c>
       <c r="C9" s="23" t="n">
@@ -4355,7 +4355,7 @@
     <row r="10">
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>Netflix</t>
+          <t>🎬 Netflix</t>
         </is>
       </c>
       <c r="C10" s="23" t="n">
@@ -4380,7 +4380,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>Spotify</t>
+          <t>🎵 Spotify</t>
         </is>
       </c>
       <c r="C11" s="23" t="n">
@@ -4405,7 +4405,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>生命保険</t>
+          <t>🛡️ 生命保険</t>
         </is>
       </c>
       <c r="C12" s="23" t="n">
@@ -4463,7 +4463,7 @@
     <row r="17">
       <c r="B17" s="38" t="inlineStr">
         <is>
-          <t>月額合計</t>
+          <t>📊 月額合計</t>
         </is>
       </c>
       <c r="C17" s="33">
@@ -4508,39 +4508,39 @@
       <c r="A3" s="14" t="n"/>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>目標名</t>
+          <t>🎯 目標名</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>目標金額</t>
+          <t>💰 目標金額</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>現在の貯蓄</t>
+          <t>📊 現在の貯蓄</t>
         </is>
       </c>
       <c r="E3" s="14" t="inlineStr">
         <is>
-          <t>残り</t>
+          <t>📉 残り</t>
         </is>
       </c>
       <c r="F3" s="14" t="inlineStr">
         <is>
-          <t>達成率</t>
+          <t>🏆 達成率</t>
         </is>
       </c>
       <c r="G3" s="14" t="inlineStr">
         <is>
-          <t>期限</t>
+          <t>📅 期限</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>緊急予備費</t>
+          <t>🆘 緊急予備費</t>
         </is>
       </c>
       <c r="C4" s="23" t="n">
@@ -4562,7 +4562,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>旅行資金</t>
+          <t>✈️ 旅行資金</t>
         </is>
       </c>
       <c r="C5" s="23" t="n">
@@ -4584,7 +4584,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>車購入</t>
+          <t>🚗 車購入</t>
         </is>
       </c>
       <c r="C6" s="23" t="n">
@@ -4606,7 +4606,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>教育資金</t>
+          <t>🎓 教育資金</t>
         </is>
       </c>
       <c r="C7" s="23" t="n">
@@ -4628,7 +4628,7 @@
     <row r="8">
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>老後資金</t>
+          <t>🏖️ 老後資金</t>
         </is>
       </c>
       <c r="C8" s="23" t="n">
@@ -4690,7 +4690,7 @@
     <row r="3">
       <c r="B3" s="38" t="inlineStr">
         <is>
-          <t>【はじめに】</t>
+          <t>📌【はじめに】</t>
         </is>
       </c>
     </row>
@@ -4714,35 +4714,35 @@
     <row r="7">
       <c r="B7" s="38" t="inlineStr">
         <is>
-          <t>【基本的な使い方】</t>
+          <t>🔰【基本的な使い方】</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>1. 各月のシートに毎日の収入と支出を記録します</t>
+          <t>1️⃣ 各月のシートに毎日の収入と支出を記録します</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>2. カテゴリごとの予算を設定します（予算列に入力）</t>
+          <t>2️⃣ カテゴリごとの予算を設定します（予算列に入力）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>3. 実績を入力すると、自動的に合計が計算されます</t>
+          <t>3️⃣ 実績を入力すると、自動的に合計が計算されます</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>4. ダッシュボードで年間のサマリーを確認できます</t>
+          <t>4️⃣ ダッシュボードで年間のサマリーを確認できます</t>
         </is>
       </c>
     </row>
@@ -4752,35 +4752,35 @@
     <row r="13">
       <c r="B13" s="38" t="inlineStr">
         <is>
-          <t>【シートの説明】</t>
+          <t>📑【シートの説明】</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>• ダッシュボード：年間の収支サマリーとグラフ</t>
+          <t>• 📊 ダッシュボード：年間の収支サマリーとグラフ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>• 1月〜12月：各月の収支管理と日別支出記録</t>
+          <t>• 📅 1月〜12月：各月の収支管理と日別支出記録</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>• 固定費・サブスク管理：毎月の固定費一覧</t>
+          <t>• 📌 固定費・サブスク管理：毎月の固定費一覧</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>• 貯蓄目標：貯蓄目標の進捗管理</t>
+          <t>• 🎯 貯蓄目標：貯蓄目標の進捗管理</t>
         </is>
       </c>
     </row>
@@ -4790,28 +4790,28 @@
     <row r="19">
       <c r="B19" s="38" t="inlineStr">
         <is>
-          <t>【カスタマイズ方法】</t>
+          <t>🔧【カスタマイズ方法】</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>• カテゴリは自由に追加・変更できます</t>
+          <t>• ✏️ カテゴリは自由に追加・変更できます</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>• 色やフォントはお好みで変更してください</t>
+          <t>• 🎨 色やフォントはお好みで変更してください</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>• 行を追加する場合は、数式が反映されるか確認してください</t>
+          <t>• ➕ 行を追加する場合は、数式が反映されるか確認してください</t>
         </is>
       </c>
     </row>
@@ -4821,35 +4821,35 @@
     <row r="24">
       <c r="B24" s="38" t="inlineStr">
         <is>
-          <t>【Tips】</t>
+          <t>💡【Tips】</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>• 毎日記録する習慣をつけましょう</t>
+          <t>• ✍️ 毎日記録する習慣をつけましょう</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>• 月初に予算を設定し、月末に振り返りをしましょう</t>
+          <t>• 🗓️ 月初に予算を設定し、月末に振り返りをしましょう</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>• 固定費は「固定費・サブスク管理」シートで一括管理</t>
+          <t>• 🔄 固定費は「固定費・サブスク管理」シートで一括管理</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>• 貯蓄目標を設定するとモチベーションが上がります</t>
+          <t>• 🚀 貯蓄目標を設定するとモチベーションが上がります</t>
         </is>
       </c>
     </row>
@@ -4859,28 +4859,28 @@
     <row r="30">
       <c r="B30" s="38" t="inlineStr">
         <is>
-          <t>【注意事項】</t>
+          <t>⚠️【注意事項】</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>• このファイルはGoogleスプレッドシートにインポートして使えます</t>
+          <t>• 🌐 このファイルはGoogleスプレッドシートにインポートして使えます</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>• 数式のあるセルを上書きしないよう注意してください</t>
+          <t>• 🔒 数式のあるセルを上書きしないよう注意してください</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>• 定期的にバックアップを取ることをおすすめします</t>
+          <t>• 💾 定期的にバックアップを取ることをおすすめします</t>
         </is>
       </c>
     </row>
@@ -4910,14 +4910,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 1月 家計簿</t>
+          <t>⛄ 1月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -4928,7 +4928,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -4943,7 +4943,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -4958,7 +4958,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -4973,7 +4973,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -4988,7 +4988,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -4999,7 +4999,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -5014,7 +5014,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -5029,7 +5029,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -5044,7 +5044,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -5059,7 +5059,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -5074,7 +5074,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -5089,7 +5089,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -5104,7 +5104,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -5119,7 +5119,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -5134,7 +5134,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -5149,7 +5149,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -5164,7 +5164,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -5179,7 +5179,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -5194,7 +5194,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -5209,14 +5209,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -5227,7 +5227,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -5238,7 +5238,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -5249,7 +5249,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -5257,27 +5257,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -5527,14 +5527,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 2月 家計簿</t>
+          <t>💝 2月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -5545,7 +5545,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -5560,7 +5560,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -5575,7 +5575,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -5590,7 +5590,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -5605,7 +5605,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -5616,7 +5616,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -5631,7 +5631,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -5646,7 +5646,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -5661,7 +5661,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -5676,7 +5676,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -5691,7 +5691,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -5706,7 +5706,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -5721,7 +5721,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -5736,7 +5736,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -5751,7 +5751,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -5766,7 +5766,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -5781,7 +5781,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -5796,7 +5796,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -5811,7 +5811,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -5826,14 +5826,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -5844,7 +5844,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -5855,7 +5855,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -5866,7 +5866,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -5874,27 +5874,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -6144,14 +6144,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 3月 家計簿</t>
+          <t>🌸 3月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -6162,7 +6162,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -6177,7 +6177,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -6192,7 +6192,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -6207,7 +6207,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -6222,7 +6222,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -6233,7 +6233,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -6248,7 +6248,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -6263,7 +6263,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -6278,7 +6278,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -6293,7 +6293,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -6308,7 +6308,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -6323,7 +6323,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -6338,7 +6338,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -6353,7 +6353,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -6368,7 +6368,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -6383,7 +6383,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -6398,7 +6398,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -6413,7 +6413,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -6428,7 +6428,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -6443,14 +6443,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -6461,7 +6461,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -6472,7 +6472,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -6483,7 +6483,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -6491,27 +6491,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -6761,14 +6761,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 4月 家計簿</t>
+          <t>🌷 4月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -6779,7 +6779,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -6794,7 +6794,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -6809,7 +6809,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -6824,7 +6824,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -6839,7 +6839,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -6850,7 +6850,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -6865,7 +6865,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -6880,7 +6880,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -6895,7 +6895,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -6910,7 +6910,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -6925,7 +6925,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -6940,7 +6940,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -6955,7 +6955,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -6970,7 +6970,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -6985,7 +6985,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -7000,7 +7000,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -7015,7 +7015,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -7030,7 +7030,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -7045,7 +7045,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -7060,14 +7060,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -7078,7 +7078,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -7089,7 +7089,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -7100,7 +7100,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -7108,27 +7108,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -7378,14 +7378,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 5月 家計簿</t>
+          <t>🎏 5月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -7396,7 +7396,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -7411,7 +7411,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -7426,7 +7426,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -7441,7 +7441,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -7456,7 +7456,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -7467,7 +7467,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -7482,7 +7482,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -7497,7 +7497,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -7512,7 +7512,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -7527,7 +7527,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -7542,7 +7542,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -7557,7 +7557,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -7572,7 +7572,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -7587,7 +7587,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -7602,7 +7602,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -7617,7 +7617,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -7632,7 +7632,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -7647,7 +7647,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -7662,7 +7662,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -7677,14 +7677,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -7695,7 +7695,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -7706,7 +7706,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -7717,7 +7717,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -7725,27 +7725,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -7995,14 +7995,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 6月 家計簿</t>
+          <t>☔ 6月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -8013,7 +8013,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -8028,7 +8028,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -8043,7 +8043,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -8058,7 +8058,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -8073,7 +8073,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -8084,7 +8084,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -8099,7 +8099,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -8114,7 +8114,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -8129,7 +8129,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -8144,7 +8144,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -8159,7 +8159,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -8174,7 +8174,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -8189,7 +8189,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -8204,7 +8204,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -8219,7 +8219,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -8234,7 +8234,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -8249,7 +8249,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -8264,7 +8264,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -8279,7 +8279,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -8294,14 +8294,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -8312,7 +8312,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -8323,7 +8323,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -8334,7 +8334,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -8342,27 +8342,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -8612,14 +8612,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 7月 家計簿</t>
+          <t>🎋 7月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -8630,7 +8630,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -8645,7 +8645,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -8660,7 +8660,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -8675,7 +8675,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -8690,7 +8690,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -8701,7 +8701,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -8716,7 +8716,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -8731,7 +8731,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -8746,7 +8746,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -8761,7 +8761,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -8776,7 +8776,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -8791,7 +8791,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -8806,7 +8806,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -8821,7 +8821,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -8836,7 +8836,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -8851,7 +8851,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -8866,7 +8866,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -8881,7 +8881,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -8896,7 +8896,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -8911,14 +8911,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -8929,7 +8929,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -8940,7 +8940,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -8951,7 +8951,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -8959,27 +8959,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>
@@ -9229,14 +9229,14 @@
     <row r="1">
       <c r="B1" s="31" t="inlineStr">
         <is>
-          <t>📋 8月 家計簿</t>
+          <t>🌻 8月 家計簿</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>【収入】</t>
+          <t>💚【収入】</t>
         </is>
       </c>
       <c r="E3" s="33">
@@ -9247,7 +9247,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>給与</t>
+          <t>💼 給与</t>
         </is>
       </c>
       <c r="C4" s="34" t="n">
@@ -9262,7 +9262,7 @@
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>副業</t>
+          <t>🔨 副業</t>
         </is>
       </c>
       <c r="C5" s="34" t="n">
@@ -9277,7 +9277,7 @@
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>投資収入</t>
+          <t>📈 投資収入</t>
         </is>
       </c>
       <c r="C6" s="34" t="n">
@@ -9292,7 +9292,7 @@
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>その他収入</t>
+          <t>🎁 その他収入</t>
         </is>
       </c>
       <c r="C7" s="34" t="n">
@@ -9307,7 +9307,7 @@
     <row r="10">
       <c r="B10" s="35" t="inlineStr">
         <is>
-          <t>【支出】</t>
+          <t>🔴【支出】</t>
         </is>
       </c>
       <c r="E10" s="33">
@@ -9318,7 +9318,7 @@
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>住居費（家賃/ローン）</t>
+          <t>🏠 住居費（家賃/ローン）</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -9333,7 +9333,7 @@
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>💡 水道光熱費</t>
         </is>
       </c>
       <c r="C12" s="34" t="n">
@@ -9348,7 +9348,7 @@
     <row r="13">
       <c r="B13" s="27" t="inlineStr">
         <is>
-          <t>食費</t>
+          <t>🍽️ 食費</t>
         </is>
       </c>
       <c r="C13" s="34" t="n">
@@ -9363,7 +9363,7 @@
     <row r="14">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>日用品</t>
+          <t>🧴 日用品</t>
         </is>
       </c>
       <c r="C14" s="34" t="n">
@@ -9378,7 +9378,7 @@
     <row r="15">
       <c r="B15" s="27" t="inlineStr">
         <is>
-          <t>交通費</t>
+          <t>🚃 交通費</t>
         </is>
       </c>
       <c r="C15" s="34" t="n">
@@ -9393,7 +9393,7 @@
     <row r="16">
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>📱 通信費</t>
         </is>
       </c>
       <c r="C16" s="34" t="n">
@@ -9408,7 +9408,7 @@
     <row r="17">
       <c r="B17" s="27" t="inlineStr">
         <is>
-          <t>保険料</t>
+          <t>🛡️ 保険料</t>
         </is>
       </c>
       <c r="C17" s="34" t="n">
@@ -9423,7 +9423,7 @@
     <row r="18">
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>医療費</t>
+          <t>🏥 医療費</t>
         </is>
       </c>
       <c r="C18" s="34" t="n">
@@ -9438,7 +9438,7 @@
     <row r="19">
       <c r="B19" s="27" t="inlineStr">
         <is>
-          <t>教育費</t>
+          <t>📚 教育費</t>
         </is>
       </c>
       <c r="C19" s="34" t="n">
@@ -9453,7 +9453,7 @@
     <row r="20">
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>🎮 娯楽費</t>
         </is>
       </c>
       <c r="C20" s="34" t="n">
@@ -9468,7 +9468,7 @@
     <row r="21">
       <c r="B21" s="27" t="inlineStr">
         <is>
-          <t>衣服費</t>
+          <t>👔 衣服費</t>
         </is>
       </c>
       <c r="C21" s="34" t="n">
@@ -9483,7 +9483,7 @@
     <row r="22">
       <c r="B22" s="27" t="inlineStr">
         <is>
-          <t>美容費</t>
+          <t>💇 美容費</t>
         </is>
       </c>
       <c r="C22" s="34" t="n">
@@ -9498,7 +9498,7 @@
     <row r="23">
       <c r="B23" s="27" t="inlineStr">
         <is>
-          <t>交際費</t>
+          <t>🍻 交際費</t>
         </is>
       </c>
       <c r="C23" s="34" t="n">
@@ -9513,7 +9513,7 @@
     <row r="24">
       <c r="B24" s="27" t="inlineStr">
         <is>
-          <t>その他</t>
+          <t>📦 その他</t>
         </is>
       </c>
       <c r="C24" s="34" t="n">
@@ -9528,14 +9528,14 @@
     <row r="27">
       <c r="B27" s="36" t="inlineStr">
         <is>
-          <t>【収支バランス】</t>
+          <t>⚖️【収支バランス】</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>収入合計</t>
+          <t>⬆️ 収入合計</t>
         </is>
       </c>
       <c r="D28" s="23">
@@ -9546,7 +9546,7 @@
     <row r="29">
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>支出合計</t>
+          <t>⬇️ 支出合計</t>
         </is>
       </c>
       <c r="D29" s="23">
@@ -9557,7 +9557,7 @@
     <row r="30">
       <c r="B30" s="37" t="inlineStr">
         <is>
-          <t>差額（貯蓄）</t>
+          <t>✨ 差額（貯蓄）</t>
         </is>
       </c>
       <c r="D30" s="23">
@@ -9568,7 +9568,7 @@
     <row r="33">
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t>【日別支出記録】</t>
+          <t>📝【日別支出記録】</t>
         </is>
       </c>
     </row>
@@ -9576,27 +9576,27 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>日付</t>
+          <t>📅 日付</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>カテゴリ</t>
+          <t>🏷️ カテゴリ</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>金額</t>
+          <t>💴 金額</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>支払方法</t>
+          <t>💳 支払方法</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>📝 メモ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance dashboard charts with axes & expand fixed costs categories
Charts:
- Bar chart (月別 収入 vs 支出): added chart title, x-axis '月', y-axis '金額（円）'
  with currency format, major gridlines, top legend, larger size (26x14),
  series fill+outline colors, gap/overlap tuning
- Line chart (月別貯蓄額): added title, both axes labels, gridlines,
  circle markers, thicker line, larger size

Bills tracker (固定費・サブスク管理):
- Expanded from 9 to 35 entries across many subcategories:
  住居 (家賃/管理費/駐車場/火災保険), 水道光熱 (電気/ガス/水道),
  通信 (携帯/ネット/NHK), 動画サブスク (Netflix/Prime/Disney+/Hulu/U-NEXT),
  音楽 (Spotify/Apple Music/YouTube Premium),
  クラウド/SW (iCloud+/Google One/M365/Adobe/ChatGPT Plus/Notion),
  保険 (生命/医療/自動車/学資), 健康 (ジム/ヨガ),
  教育 (英会話/新聞), 交通 (定期券), その他 (年会費/ふるさと納税)
- Each entry has an icon, payment method, category, and status

Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/a9ee436f-8b93-4661-94c0-b2945aa8fee1

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -322,8 +322,23 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="11"/>
   <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>月別 収入 vs 支出 推移</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
     <plotArea>
       <barChart>
         <barDir val="col"/>
@@ -341,9 +356,15 @@
               <a:srgbClr val="27AE60"/>
             </a:solidFill>
             <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="27AE60"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <showVal val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'ダッシュボード'!$B$10:$B$21</f>
@@ -368,9 +389,15 @@
               <a:srgbClr val="E74C3C"/>
             </a:solidFill>
             <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E74C3C"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <showVal val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'ダッシュボード'!$B$10:$B$21</f>
@@ -382,7 +409,8 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <gapWidth val="80"/>
+        <overlap val="-10"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -391,7 +419,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>月</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -402,6 +446,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -419,14 +464,14 @@
             </rich>
           </tx>
         </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <numFmt formatCode="#,##0&quot;円&quot;" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -436,8 +481,23 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+  <style val="12"/>
   <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>月別貯蓄額の推移</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
     <plotArea>
       <lineChart>
         <grouping val="standard"/>
@@ -450,7 +510,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="30000">
               <a:solidFill>
                 <a:srgbClr val="3498DB"/>
               </a:solidFill>
@@ -458,8 +518,12 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="8"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="3498DB"/>
+              </a:solidFill>
               <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -484,7 +548,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>月</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -495,6 +575,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -512,14 +593,14 @@
             </rich>
           </tx>
         </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <numFmt formatCode="#,##0&quot;円&quot;" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -594,7 +675,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3960000"/>
+    <ext cx="9360000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -616,7 +697,7 @@
       <row>41</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3600000"/>
+    <ext cx="9360000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -4144,7 +4225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4205,7 +4286,7 @@
     <row r="4">
       <c r="B4" s="27" t="inlineStr">
         <is>
-          <t>🏠 家賃</t>
+          <t>🏠 家賃 / 住宅ローン</t>
         </is>
       </c>
       <c r="C4" s="23" t="n">
@@ -4225,19 +4306,23 @@
         </is>
       </c>
       <c r="G4" s="27" t="inlineStr"/>
-      <c r="H4" s="27" t="inlineStr"/>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>⚡ 電気代</t>
+          <t>🏢 管理費・共益費</t>
         </is>
       </c>
       <c r="C5" s="23" t="n">
         <v>8000</v>
       </c>
       <c r="D5" s="27" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
@@ -4246,23 +4331,27 @@
       </c>
       <c r="F5" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>住居費</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr"/>
-      <c r="H5" s="27" t="inlineStr"/>
+      <c r="H5" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>🔥 ガス代</t>
+          <t>🅿️ 駐車場代</t>
         </is>
       </c>
       <c r="C6" s="23" t="n">
-        <v>5000</v>
+        <v>12000</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
@@ -4271,23 +4360,27 @@
       </c>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>住居費</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr"/>
-      <c r="H6" s="27" t="inlineStr"/>
+      <c r="H6" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>💧 水道代</t>
+          <t>🏘️ 火災・地震保険</t>
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
@@ -4296,98 +4389,114 @@
       </c>
       <c r="F7" s="27" t="inlineStr">
         <is>
-          <t>水道光熱費</t>
+          <t>保険料</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr"/>
-      <c r="H7" s="27" t="inlineStr"/>
+      <c r="H7" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>📱 携帯電話</t>
+          <t>⚡ 電気代</t>
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="D8" s="27" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>クレジットカード</t>
+          <t>口座振替</t>
         </is>
       </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>水道光熱費</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr"/>
-      <c r="H8" s="27" t="inlineStr"/>
+      <c r="H8" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="27" t="inlineStr">
         <is>
-          <t>🌐 インターネット</t>
+          <t>🔥 ガス代</t>
         </is>
       </c>
       <c r="C9" s="23" t="n">
         <v>5000</v>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E9" s="27" t="inlineStr">
         <is>
-          <t>クレジットカード</t>
+          <t>口座振替</t>
         </is>
       </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
-          <t>通信費</t>
+          <t>水道光熱費</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr"/>
-      <c r="H9" s="27" t="inlineStr"/>
+      <c r="H9" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="27" t="inlineStr">
         <is>
-          <t>🎬 Netflix</t>
+          <t>💧 水道代</t>
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>1490</v>
+        <v>4000</v>
       </c>
       <c r="D10" s="27" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E10" s="27" t="inlineStr">
         <is>
-          <t>クレジットカード</t>
+          <t>口座振替</t>
         </is>
       </c>
       <c r="F10" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>水道光熱費</t>
         </is>
       </c>
       <c r="G10" s="27" t="inlineStr"/>
-      <c r="H10" s="27" t="inlineStr"/>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="27" t="inlineStr">
         <is>
-          <t>🎵 Spotify</t>
+          <t>📱 携帯電話</t>
         </is>
       </c>
       <c r="C11" s="23" t="n">
-        <v>980</v>
+        <v>5000</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E11" s="27" t="inlineStr">
         <is>
@@ -4396,78 +4505,840 @@
       </c>
       <c r="F11" s="27" t="inlineStr">
         <is>
-          <t>娯楽費</t>
+          <t>通信費</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr"/>
-      <c r="H11" s="27" t="inlineStr"/>
+      <c r="H11" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="27" t="inlineStr">
         <is>
+          <t>🌐 インターネット回線</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>通信費</t>
+        </is>
+      </c>
+      <c r="G12" s="27" t="inlineStr"/>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>📡 NHK受信料</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>1275</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>通信費</t>
+        </is>
+      </c>
+      <c r="G13" s="27" t="inlineStr"/>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="27" t="inlineStr">
+        <is>
+          <t>🎬 Netflix</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>1490</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="inlineStr"/>
+      <c r="H14" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="27" t="inlineStr">
+        <is>
+          <t>🎞️ Amazon Prime</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>600</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="inlineStr"/>
+      <c r="H15" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="27" t="inlineStr">
+        <is>
+          <t>📺 Disney+</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>990</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G16" s="27" t="inlineStr"/>
+      <c r="H16" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t>🎥 Hulu</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>1026</v>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="inlineStr"/>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t>📼 U-NEXT</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>2189</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="inlineStr"/>
+      <c r="H18" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="27" t="inlineStr">
+        <is>
+          <t>🎵 Spotify</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>980</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G19" s="27" t="inlineStr"/>
+      <c r="H19" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="27" t="inlineStr">
+        <is>
+          <t>🎧 Apple Music</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D20" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G20" s="27" t="inlineStr"/>
+      <c r="H20" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="27" t="inlineStr">
+        <is>
+          <t>📻 YouTube Premium</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>1280</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="inlineStr">
+        <is>
+          <t>娯楽費</t>
+        </is>
+      </c>
+      <c r="G21" s="27" t="inlineStr"/>
+      <c r="H21" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="27" t="inlineStr">
+        <is>
+          <t>☁️ iCloud+ ストレージ</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>400</v>
+      </c>
+      <c r="D22" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>通信費</t>
+        </is>
+      </c>
+      <c r="G22" s="27" t="inlineStr"/>
+      <c r="H22" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>📁 Google One</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>250</v>
+      </c>
+      <c r="D23" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>通信費</t>
+        </is>
+      </c>
+      <c r="G23" s="27" t="inlineStr"/>
+      <c r="H23" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>💼 Microsoft 365</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>1284</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>通信費</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr"/>
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>🎨 Adobe Creative Cloud</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="n">
+        <v>6480</v>
+      </c>
+      <c r="D25" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="inlineStr">
+        <is>
+          <t>教育費</t>
+        </is>
+      </c>
+      <c r="G25" s="27" t="inlineStr"/>
+      <c r="H25" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>🤖 ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D26" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="inlineStr">
+        <is>
+          <t>教育費</t>
+        </is>
+      </c>
+      <c r="G26" s="27" t="inlineStr"/>
+      <c r="H26" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>📔 Notion</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D27" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="inlineStr">
+        <is>
+          <t>教育費</t>
+        </is>
+      </c>
+      <c r="G27" s="27" t="inlineStr"/>
+      <c r="H27" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="27" t="inlineStr">
+        <is>
           <t>🛡️ 生命保険</t>
         </is>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C28" s="23" t="n">
         <v>10000</v>
       </c>
-      <c r="D12" s="27" t="n">
+      <c r="D28" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="E12" s="27" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>口座振替</t>
         </is>
       </c>
-      <c r="F12" s="27" t="inlineStr">
+      <c r="F28" s="27" t="inlineStr">
         <is>
           <t>保険料</t>
         </is>
       </c>
-      <c r="G12" s="27" t="inlineStr"/>
-      <c r="H12" s="27" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="27" t="inlineStr"/>
-      <c r="C13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="27" t="inlineStr"/>
-      <c r="E13" s="27" t="inlineStr"/>
-      <c r="F13" s="27" t="inlineStr"/>
-      <c r="G13" s="27" t="inlineStr"/>
-      <c r="H13" s="27" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="27" t="inlineStr"/>
-      <c r="C14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="27" t="inlineStr"/>
-      <c r="E14" s="27" t="inlineStr"/>
-      <c r="F14" s="27" t="inlineStr"/>
-      <c r="G14" s="27" t="inlineStr"/>
-      <c r="H14" s="27" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="27" t="inlineStr"/>
-      <c r="C15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="27" t="inlineStr"/>
-      <c r="E15" s="27" t="inlineStr"/>
-      <c r="F15" s="27" t="inlineStr"/>
-      <c r="G15" s="27" t="inlineStr"/>
-      <c r="H15" s="27" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="38" t="inlineStr">
+      <c r="G28" s="27" t="inlineStr"/>
+      <c r="H28" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>🏥 医療保険</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="inlineStr">
+        <is>
+          <t>保険料</t>
+        </is>
+      </c>
+      <c r="G29" s="27" t="inlineStr"/>
+      <c r="H29" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>🚗 自動車保険</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>保険料</t>
+        </is>
+      </c>
+      <c r="G30" s="27" t="inlineStr"/>
+      <c r="H30" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>👨‍👩‍👧 学資保険</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <v>27</v>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="inlineStr">
+        <is>
+          <t>保険料</t>
+        </is>
+      </c>
+      <c r="G31" s="27" t="inlineStr"/>
+      <c r="H31" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>💪 ジム会費</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="inlineStr">
+        <is>
+          <t>美容費</t>
+        </is>
+      </c>
+      <c r="G32" s="27" t="inlineStr"/>
+      <c r="H32" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>🧘 ヨガスタジオ</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="inlineStr">
+        <is>
+          <t>美容費</t>
+        </is>
+      </c>
+      <c r="G33" s="27" t="inlineStr"/>
+      <c r="H33" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>📚 英会話レッスン</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="inlineStr">
+        <is>
+          <t>教育費</t>
+        </is>
+      </c>
+      <c r="G34" s="27" t="inlineStr"/>
+      <c r="H34" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>📖 新聞購読</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>4400</v>
+      </c>
+      <c r="D35" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="inlineStr">
+        <is>
+          <t>教育費</t>
+        </is>
+      </c>
+      <c r="G35" s="27" t="inlineStr"/>
+      <c r="H35" s="27" t="inlineStr">
+        <is>
+          <t>停止中</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>🚃 定期券</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D36" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="inlineStr">
+        <is>
+          <t>交通費</t>
+        </is>
+      </c>
+      <c r="G36" s="27" t="inlineStr"/>
+      <c r="H36" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>💳 クレジットカード年会費</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>11000</v>
+      </c>
+      <c r="D37" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>口座振替</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G37" s="27" t="inlineStr"/>
+      <c r="H37" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>🎁 ふるさと納税（積立）</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D38" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="E38" s="27" t="inlineStr">
+        <is>
+          <t>クレジットカード</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="G38" s="27" t="inlineStr"/>
+      <c r="H38" s="27" t="inlineStr">
+        <is>
+          <t>継続中</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="27" t="inlineStr"/>
+      <c r="C39" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="27" t="inlineStr"/>
+      <c r="E39" s="27" t="inlineStr"/>
+      <c r="F39" s="27" t="inlineStr"/>
+      <c r="G39" s="27" t="inlineStr"/>
+      <c r="H39" s="27" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="27" t="inlineStr"/>
+      <c r="C40" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="27" t="inlineStr"/>
+      <c r="E40" s="27" t="inlineStr"/>
+      <c r="F40" s="27" t="inlineStr"/>
+      <c r="G40" s="27" t="inlineStr"/>
+      <c r="H40" s="27" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="27" t="inlineStr"/>
+      <c r="C41" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="27" t="inlineStr"/>
+      <c r="E41" s="27" t="inlineStr"/>
+      <c r="F41" s="27" t="inlineStr"/>
+      <c r="G41" s="27" t="inlineStr"/>
+      <c r="H41" s="27" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="38" t="inlineStr">
         <is>
           <t>📊 月額合計</t>
         </is>
       </c>
-      <c r="C17" s="33">
-        <f>SUM(C4:C15)</f>
+      <c r="C43" s="33">
+        <f>SUM(C4:C41)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add dropdown validation for category/payment in daily expense log
- Category column: dropdown with all 14 expense categories
- Payment method column: dropdown (現金/クレジットカード/デビット/電子マネー/QR/口座振替/その他)
- Column headers made more descriptive: 日付→日付（何日）, カテゴリ→カテゴリ（種類）, 金額→金額（円）, メモ→メモ・備考

Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/36b6d8af-ca16-4df9-a9eb-ef0a2298866a

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -2119,17 +2119,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -2364,6 +2364,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2736,17 +2744,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -2756,7 +2764,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -2981,6 +2989,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3353,17 +3369,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -3373,7 +3389,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -3598,6 +3614,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3970,17 +3994,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -3990,7 +4014,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -4215,6 +4239,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6128,17 +6160,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -6148,7 +6180,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -6373,6 +6405,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6745,17 +6785,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -6765,7 +6805,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -6990,6 +7030,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7362,17 +7410,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -7382,7 +7430,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -7607,6 +7655,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7979,17 +8035,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -7999,7 +8055,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -8224,6 +8280,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8596,17 +8660,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -8616,7 +8680,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -8841,6 +8905,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9213,17 +9285,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -9233,7 +9305,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -9458,6 +9530,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9830,17 +9910,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -9850,7 +9930,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -10075,6 +10155,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10447,17 +10535,17 @@
       <c r="A34" s="14" t="n"/>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>📅 日付</t>
+          <t>📅 日付（何日）</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ</t>
+          <t>🏷️ カテゴリ（種類）</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>💴 金額</t>
+          <t>💴 金額（円）</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -10467,7 +10555,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>📝 メモ</t>
+          <t>📝 メモ・備考</t>
         </is>
       </c>
     </row>
@@ -10692,6 +10780,14 @@
   <mergeCells count="1">
     <mergeCell ref="B1:F1"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
+      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
+      <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change daily expense dropdown from category to item names
- Column header: カテゴリ（種類）→ 項目名
- Dropdown options: specific item names (家賃, 電気代, 食料品, 外食, etc.)
- Added EXPENSE_ITEMS list with 31 common expense items

Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/c09a2e77-df75-4c93-b6dc-35947d053e08

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -2124,7 +2124,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -2365,8 +2365,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -2990,8 +2990,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -3615,8 +3615,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -4240,8 +4240,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -6406,8 +6406,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -6790,7 +6790,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -7031,8 +7031,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -7656,8 +7656,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -8040,7 +8040,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -8281,8 +8281,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -8906,8 +8906,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -9531,8 +9531,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -9915,7 +9915,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -10156,8 +10156,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>
@@ -10540,7 +10540,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>🏷️ カテゴリ（種類）</t>
+          <t>📋 項目名</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -10781,8 +10781,8 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="カテゴリエラー" error="リストからカテゴリを選択してください" promptTitle="カテゴリ選択" prompt="カテゴリを選んでください" type="list">
-      <formula1>"住居費（家賃/ローン）,水道光熱費,食費,日用品,交通費,通信費,保険料,医療費,教育費,娯楽費,衣服費,美容費,交際費,その他"</formula1>
+    <dataValidation sqref="C35:C65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="項目名エラー" error="リストから項目名を選択してください" promptTitle="項目名選択" prompt="項目名を選んでください" type="list">
+      <formula1>"家賃,管理費,駐車場代,電気代,ガス代,水道代,食料品,外食,カフェ,日用品,消耗品,電車,バス,タクシー,ガソリン,携帯電話,ネット回線,Netflix,Spotify,YouTube,保険料,医療費,薬代,書籍,習い事,衣服,美容院,飲み会,ご祝儀,コンビニ,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="E35:E65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="支払方法エラー" error="リストから支払方法を選択してください" promptTitle="支払方法選択" prompt="支払方法を選んでください" type="list">
       <formula1>"現金,クレジットカード,デビットカード,電子マネー,QRコード決済,口座振替,その他"</formula1>

</xml_diff>

<commit_message>
Change all fonts from Arial to メイリオ (Meiryo) for softer Japanese typography
Agent-Logs-Url: https://github.com/yyappyyy/app-cowork/sessions/f127cefe-d30e-423b-b0e3-bc10baa550a4

Co-authored-by: yyappyyy <27191505+yyappyyy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/household-budget-spreadsheet/家計簿テンプレート.xlsx
+++ b/household-budget-spreadsheet/家計簿テンプレート.xlsx
@@ -44,65 +44,65 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="002C3E50"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="0027AE60"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="00E74C3C"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="003498DB"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="002C3E50"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="002C3E50"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="002C3E50"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="メイリオ"/>
       <b val="1"/>
       <color rgb="002C3E50"/>
       <sz val="11"/>

</xml_diff>